<commit_message>
Improve good conduct closing text photo processing and Excel template
</commit_message>
<xml_diff>
--- a/Good Conduct Data Template.xlsx
+++ b/Good Conduct Data Template.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:Z2"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -427,8 +427,6 @@
     <col min="24" max="24" width="22.83203125" customWidth="1"/>
     <col min="25" max="25" width="22.83203125" customWidth="1"/>
     <col min="26" max="26" width="22.83203125" customWidth="1"/>
-    <col min="27" max="27" width="22.83203125" customWidth="1"/>
-    <col min="28" max="28" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -510,43 +508,37 @@
       <c r="Z1" t="str">
         <v>expiryEn</v>
       </c>
-      <c r="AA1" t="str">
-        <v>notesAr</v>
-      </c>
-      <c r="AB1" t="str">
-        <v>notesEn</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>11/12/2025</v>
+        <v/>
       </c>
       <c r="B2" t="str">
-        <v>جميل جبر أحمد</v>
+        <v/>
       </c>
       <c r="C2" t="str">
-        <v>Jameel Jabr Ahmed</v>
+        <v/>
       </c>
       <c r="D2" t="str">
-        <v>الرملي</v>
+        <v/>
       </c>
       <c r="E2" t="str">
-        <v>Al Ramli</v>
+        <v/>
       </c>
       <c r="F2" t="str">
-        <v>16/02/1995</v>
+        <v/>
       </c>
       <c r="G2" t="str">
-        <v>السعودية، جدة</v>
+        <v/>
       </c>
       <c r="H2" t="str">
-        <v>Jeddah, Saudi Arabia</v>
+        <v/>
       </c>
       <c r="I2" t="str">
-        <v>اليمن</v>
+        <v/>
       </c>
       <c r="J2" t="str">
-        <v>Yemen</v>
+        <v/>
       </c>
       <c r="K2" t="str">
         <v>جواز سفر</v>
@@ -555,64 +547,58 @@
         <v>Passport</v>
       </c>
       <c r="M2" t="str">
-        <v>10878313</v>
+        <v/>
       </c>
       <c r="N2" t="str">
-        <v>10878313</v>
+        <v/>
       </c>
       <c r="O2" t="str">
-        <v>11/03/2026</v>
+        <v/>
       </c>
       <c r="P2" t="str">
-        <v>11/03/2026</v>
+        <v/>
       </c>
       <c r="Q2" t="str">
-        <v>منسوب مبيعات</v>
+        <v/>
       </c>
       <c r="R2" t="str">
-        <v>Sales Representative</v>
+        <v/>
       </c>
       <c r="S2" t="str">
-        <v>01/03/2023</v>
+        <v/>
       </c>
       <c r="T2" t="str">
-        <v>01/03/2023</v>
+        <v/>
       </c>
       <c r="U2" t="str">
-        <v>معين</v>
+        <v/>
       </c>
       <c r="V2" t="str">
-        <v>Ma'in</v>
+        <v/>
       </c>
       <c r="W2" t="str">
-        <v>سفارة عمان</v>
+        <v/>
       </c>
       <c r="X2" t="str">
-        <v>Embassy of Oman</v>
+        <v/>
       </c>
       <c r="Y2" t="str">
-        <v>11/03/2026</v>
+        <v/>
       </c>
       <c r="Z2" t="str">
-        <v>11/03/2026</v>
-      </c>
-      <c r="AA2" t="str">
-        <v>تم التحقق من سجلاتنا.</v>
-      </c>
-      <c r="AB2" t="str">
-        <v>OUR RECORDS HAVE BEEN VERIFIED.</v>
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A8"/>
   <cols>
     <col min="1" max="1" width="120.83203125" customWidth="1"/>
   </cols>
@@ -629,34 +615,44 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>تواريخ Excel: استخدم DD/MM/YYYY أو YYYY-MM-DD.</v>
+        <v>تاريخ الإصدار هو تاريخ إصدار وثيقة حسن السيرة والسلوك، وليس تاريخ إصدار جواز أو بطاقة الشخص.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>الأرقام النظامية issueNo و referenceNo و internalNo و issuanceNo لا تكتبها؛ ينشئها النظام بعد الاستيراد.</v>
+        <v>أدخل بيانات الشخص الفعلية في الحقول المطابقة لها، واترك الملاحظات خارج القالب لأن الجملة الخاتمية ثابتة في النظام.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>الصورة تُرفع من داخل النظام وليست داخل ملف Excel.</v>
+        <v>تواريخ Excel: استخدم DD/MM/YYYY أو YYYY-MM-DD.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>الأرقام النظامية issueNo و referenceNo و internalNo و issuanceNo لا تكتبها؛ ينشئها النظام بعد الاستيراد.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>الصورة تُرفع من داخل النظام وليست داخل ملف Excel.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
         <v>لا تغيّر أسماء أعمدة ورقة Good Conduct حتى يتم الاستيراد بشكل صحيح.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A8"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D28"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -1044,49 +1040,21 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>notesAr</v>
+        <v>issueNo / referenceNo / internalNo / issuanceNo</v>
       </c>
       <c r="B28" t="str">
-        <v>الملاحظة</v>
+        <v>أرقام النظام</v>
       </c>
       <c r="C28" t="str">
-        <v>Notes</v>
+        <v>System identifiers</v>
       </c>
       <c r="D28" t="str">
-        <v>بيانات مستخدم قابلة للاستيراد</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v>notesEn</v>
-      </c>
-      <c r="B29" t="str">
-        <v>الملاحظة بالإنجليزي</v>
-      </c>
-      <c r="C29" t="str">
-        <v>Notes (English)</v>
-      </c>
-      <c r="D29" t="str">
-        <v>بيانات مستخدم قابلة للاستيراد</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v>issueNo / referenceNo / internalNo / issuanceNo</v>
-      </c>
-      <c r="B30" t="str">
-        <v>أرقام النظام</v>
-      </c>
-      <c r="C30" t="str">
-        <v>System identifiers</v>
-      </c>
-      <c r="D30" t="str">
         <v>لا تعبئها؛ ينشئها النظام بعد الاستيراد</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D28"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>